<commit_message>
Update reports 2026-09-10 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-10.xlsx
+++ b/gex_pivot_levels_2026-09-10.xlsx
@@ -639,12 +639,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$12.00M</t>
+          <t>-$12.89M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$20.43M</t>
+          <t>+$21.96M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$2.14M</t>
+          <t>-$2.24M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$3.13M</t>
+          <t>+$3.27M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$6.64M</t>
+          <t>-$6.99M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$8.12M</t>
+          <t>+$8.54M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -771,12 +771,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$1.44M</t>
+          <t>-$1.54M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$17.90M</t>
+          <t>+$19.10M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>+$1.13M</t>
+          <t>+$1.18M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$19.00M</t>
+          <t>+$19.92M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$3.45M</t>
+          <t>+$3.61M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$14.73M</t>
+          <t>+$15.41M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -924,12 +924,12 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>+$14.45M</t>
+          <t>+$14.10M</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>+$28.49M</t>
+          <t>+$27.81M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>+$5.04M</t>
+          <t>+$4.61M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$23.19M</t>
+          <t>+$21.23M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>+$6.03M</t>
+          <t>+$5.11M</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>+$8.99M</t>
+          <t>+$7.61M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -3207,12 +3207,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>+$14.45M</t>
+          <t>+$14.10M</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>+$28.49M</t>
+          <t>+$27.81M</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -3265,38 +3265,42 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>7719.39</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>+$5.04M</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>+$23.19M</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="B4" s="5" t="n">
+        <v>7631.71</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>760</v>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-$15.29M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>+$22.63M</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3305,24 +3309,24 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7631.71</v>
+        <v>7619.39</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>760</v>
+        <v>7600</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>-$15.29M</t>
+          <t>-$12.89M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>+$22.63M</t>
+          <t>+$21.96M</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -3337,42 +3341,38 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
-        <v>7619.39</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="B6" s="2" t="n">
+        <v>7719.39</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>7700</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>-$12.00M</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>+$20.43M</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>+$4.61M</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>+$21.23M</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3431,12 +3431,12 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>+$1.13M</t>
+          <t>+$1.18M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>+$19.00M</t>
+          <t>+$19.92M</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>-$1.44M</t>
+          <t>-$1.54M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>+$17.90M</t>
+          <t>+$19.10M</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3553,76 +3553,76 @@
       <c r="H11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>7679.39</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>7660</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>+$3.61M</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>+$15.41M</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B13" s="5" t="n">
         <v>4520.38</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C13" s="5" t="n">
         <v>101</v>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>+$14.44M</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>+$14.80M</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>7679.39</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>7660</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>+$3.45M</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>+$14.73M</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3887,72 +3887,76 @@
       <c r="H20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
-        <v>7744.39</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>7725</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>+$6.03M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>+$8.99M</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
+      <c r="B21" s="5" t="n">
+        <v>7581.63</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>755</v>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>-$6.53M</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>+$8.97M</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
-        <v>7581.63</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>755</v>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="B22" s="2" t="n">
+        <v>7721.86</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>769</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>-$6.53M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>+$8.97M</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>+$1.45M</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>+$8.84M</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3965,24 +3969,24 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>7721.86</v>
+        <v>7639.39</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>769</v>
+        <v>7620</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>+$1.45M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>-$6.99M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+$8.84M</t>
+          <t>+$8.54M</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -3997,80 +4001,76 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>29781.43</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>725</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>+$5.52M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>+$7.94M</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>7639.39</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>7620</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="B25" s="2" t="n">
+        <v>7744.39</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7725</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>-$6.64M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>+$8.12M</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>29781.43</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>725</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>+$5.52M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>+$7.94M</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$5.11M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>+$7.61M</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -4519,28 +4519,28 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>2927.46</v>
+        <v>7624.39</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>291</v>
+        <v>7605</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>-$2.14M</t>
+          <t>-$2.24M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$3.14M</t>
+          <t>+$3.27M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -4557,18 +4557,18 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>7624.39</v>
+        <v>2927.46</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>7605</v>
+        <v>291</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>+$3.13M</t>
+          <t>+$3.14M</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">

</xml_diff>